<commit_message>
Replace crude native charts with clear labeled charts (matplotlib)
Every bar labeled with its value and category:
- Chart 1: the $700 credit across first 7 orders (refunds the qual, then stops)
- Chart 2: total annual account cost, all options, CJB towering ~10x
- Chart 3: realistic SNP-vs-Market view with the redundancy premium called out
Embedded as images in a new Charts tab and on the data tabs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Cost_Scenarios.xlsx
+++ b/PVA second supplier initiative/PVA_Cost_Scenarios.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inputs &amp; Sources" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Per-Order (credit)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Annual Scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Market Research" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Charts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inputs &amp; Sources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Per-Order (credit)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Annual Scenarios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Market Research" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,6 +101,12 @@
       <color rgb="00404040"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="15"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -165,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -231,6 +238,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -307,332 +315,88 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>CJB cost per order — credit applies to first 7 only</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Per-Order (credit)'!C5</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Per-Order (credit)'!$B$6:$B$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Per-Order (credit)'!$C$6:$C$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Per-Order (credit)'!D5</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Per-Order (credit)'!$B$6:$B$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Per-Order (credit)'!$D$6:$D$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Order #</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>$ per order (drum)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="14725650" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="17316450" cy="8096250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>66</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15611475" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Total annual account cost — all options</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Annual Scenarios'!C5</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Annual Scenarios'!$B$6:$B$12</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Annual Scenarios'!$C$6:$C$12</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>$ / year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Realistic options — SNP baseline vs Market (2nd source)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Annual Scenarios'!C17</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Annual Scenarios'!$B$18:$B$20</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Annual Scenarios'!$C$18:$C$20</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>$ / year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -640,26 +404,141 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="15525750" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="14725650" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="14725650" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="14725650" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="14725650" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -667,41 +546,271 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="17316450" cy="8096250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="15611475" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="17316450" cy="8096250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15611475" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="17316450" cy="8096250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15611475" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="17316450" cy="8096250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15611475" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="17316450" cy="8096250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15611475" cy="7810500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -996,6 +1105,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="33" t="inlineStr">
+        <is>
+          <t>PVA Second Source — Cost Charts</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Every bar is labeled. See data tabs for the underlying numbers and the Market Research tab for sources.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1245,7 +1383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1457,7 +1595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1622,7 +1760,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Switch front scenario charts to high-end market rate ($2.55/lb)
Charts 2 and 3 and the Annual Scenarios data now use the high-end market
rate per request (Market @25% $81k, @35% $93k). Chart 1 (credit) unchanged.
Full low/base/high range remains documented on the Market Research tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Cost_Scenarios.xlsx
+++ b/PVA second supplier initiative/PVA_Cost_Scenarios.xlsx
@@ -349,7 +349,7 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17316450" cy="8096250"/>
+    <ext cx="20726400" cy="8096250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -374,7 +374,7 @@
       <row>66</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15611475" cy="7810500"/>
+    <ext cx="17021175" cy="7810500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -404,7 +404,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15525750" cy="7810500"/>
+    <ext cx="14725650" cy="7810500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -446,90 +446,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="14725650" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="14725650" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="14725650" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -546,7 +462,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17316450" cy="8096250"/>
+    <ext cx="20726400" cy="8096250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -574,7 +490,7 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15611475" cy="7810500"/>
+    <ext cx="17021175" cy="7810500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -602,7 +518,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17316450" cy="8096250"/>
+    <ext cx="20726400" cy="8096250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -610,174 +526,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15611475" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="17316450" cy="8096250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15611475" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="17316450" cy="8096250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15611475" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="17316450" cy="8096250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -795,14 +543,14 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15611475" cy="7810500"/>
+    <ext cx="17021175" cy="7810500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1648,21 +1396,21 @@
     <row r="7">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Market @25%</t>
+          <t>Market (high $2.55) @25%</t>
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>61685</v>
+        <v>81120</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Market @35%</t>
+          <t>Market (high $2.55) @35%</t>
         </is>
       </c>
       <c r="C8" s="19" t="n">
-        <v>66079</v>
+        <v>93288</v>
       </c>
     </row>
     <row r="9">
@@ -1737,21 +1485,21 @@
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Market @25%</t>
+          <t>Market (high $2.55) @25%</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
-        <v>61685</v>
+        <v>81120</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Market @35%</t>
+          <t>Market (high $2.55) @35%</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>66079</v>
+        <v>93288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reframe graphs to show EXTRA cost (redundancy premium), not SNP-inclusive totals
- Chart 2: extra $/yr vs all-SNP for market(high) and CJB at 25%/35%.
- Chart 3: market extra by low/base/high rate at 25%/35% — shows the range
  (base ~$15k, high ~$43k at 35%) so the premium is in context.
- Annual tab: added 'EXTRA vs all-SNP' column as the decision number.
Estimates re-verified; the prior totals were correct but included the SNP
spend incurred either way.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Cost_Scenarios.xlsx
+++ b/PVA second supplier initiative/PVA_Cost_Scenarios.xlsx
@@ -82,13 +82,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
     <font>
@@ -172,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -205,22 +205,31 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -232,8 +241,8 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -349,7 +358,7 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="20726400" cy="8096250"/>
+    <ext cx="17392650" cy="6953250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -374,7 +383,7 @@
       <row>66</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17021175" cy="7810500"/>
+    <ext cx="16021050" cy="7810500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -418,34 +427,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="14725650" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -462,7 +443,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="20726400" cy="8096250"/>
+    <ext cx="17392650" cy="6953250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -470,62 +451,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="17021175" cy="7810500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="20726400" cy="8096250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -543,14 +468,14 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17021175" cy="7810500"/>
+    <ext cx="16021050" cy="7810500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -857,7 +782,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="33" t="inlineStr">
+      <c r="B2" s="36" t="inlineStr">
         <is>
           <t>PVA Second Source — Cost Charts</t>
         </is>
@@ -1349,12 +1274,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C20"/>
+  <dimension ref="B2:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1379,7 +1305,12 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Annual $</t>
+          <t>Total account $/yr</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>EXTRA vs all-SNP $/yr</t>
         </is>
       </c>
     </row>
@@ -1392,69 +1323,97 @@
       <c r="C6" s="17" t="n">
         <v>50700</v>
       </c>
+      <c r="D6" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Market (high $2.55) @25%</t>
         </is>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="20" t="n">
         <v>81120</v>
       </c>
+      <c r="D7" s="21" t="n">
+        <v>30420</v>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Market (high $2.55) @35%</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="20" t="n">
         <v>93288</v>
       </c>
+      <c r="D8" s="21" t="n">
+        <v>42588</v>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>CJB @25% — Yr 1 (credit)</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="23" t="n">
         <v>175367</v>
       </c>
+      <c r="D9" s="24" t="n">
+        <v>124667</v>
+      </c>
     </row>
     <row r="10">
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>CJB @25% — Yr 2+</t>
         </is>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="23" t="n">
         <v>180267</v>
       </c>
+      <c r="D10" s="24" t="n">
+        <v>129567</v>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>CJB @35% — Yr 1 (credit)</t>
         </is>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="23" t="n">
         <v>227193</v>
       </c>
+      <c r="D11" s="24" t="n">
+        <v>176493</v>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>CJB @35% — Yr 2+</t>
         </is>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="23" t="n">
         <v>232093</v>
       </c>
+      <c r="D12" s="24" t="n">
+        <v>181393</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>EXTRA = the redundancy premium (what dual-sourcing ADDS). The drums are bought either way, so this is the real decision number.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>Realistic options only (CJB excluded — it is ~10x and dwarfs the scale)</t>
         </is>
@@ -1478,7 +1437,7 @@
           <t>All-SNP baseline</t>
         </is>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="26" t="n">
         <v>50700</v>
       </c>
     </row>
@@ -1488,7 +1447,7 @@
           <t>Market (high $2.55) @25%</t>
         </is>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="26" t="n">
         <v>81120</v>
       </c>
     </row>
@@ -1498,7 +1457,7 @@
           <t>Market (high $2.55) @35%</t>
         </is>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="26" t="n">
         <v>93288</v>
       </c>
     </row>
@@ -1550,17 +1509,17 @@
       <c r="E5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>BASE</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1572,13 +1531,13 @@
           <t>all-in $/lb finished</t>
         </is>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="28" t="n">
         <v>0.85</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="28" t="n">
         <v>1.4</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="28" t="n">
         <v>2.55</v>
       </c>
     </row>
@@ -1588,13 +1547,13 @@
           <t xml:space="preserve">  = per 450-lb drum</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="29" t="n">
         <v>382</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="D8" s="29" t="n">
         <v>630</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E8" s="29" t="n">
         <v>1148</v>
       </c>
     </row>
@@ -1604,13 +1563,13 @@
           <t xml:space="preserve">  vs SNP $0.75/lb</t>
         </is>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="30" t="n">
         <v>1.133333333333333</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="30" t="n">
         <v>1.866666666666666</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="30" t="n">
         <v>3.4</v>
       </c>
     </row>
@@ -1620,17 +1579,17 @@
           <t>BOTTOM-UP BUILD (per lb finished)</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>BASE</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1642,13 +1601,13 @@
           <t>Raw material (resin ~$1.52/lb x ~11%)</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="31" t="n">
         <v>0.16</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="31" t="n">
         <v>0.18</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="31" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1658,13 +1617,13 @@
           <t>Conversion (labor $40/hr + QC + margin)</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="31" t="n">
         <v>0.47</v>
       </c>
-      <c r="D13" s="28" t="n">
+      <c r="D13" s="31" t="n">
         <v>0.85</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E13" s="31" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -1674,169 +1633,169 @@
           <t>Freight (1-drum LTL, regional)</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="31" t="n">
         <v>0.22</v>
       </c>
-      <c r="D14" s="28" t="n">
+      <c r="D14" s="31" t="n">
         <v>0.37</v>
       </c>
-      <c r="E14" s="28" t="n">
+      <c r="E14" s="31" t="n">
         <v>0.55</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>ALL-IN $/lb</t>
         </is>
       </c>
-      <c r="C15" s="30" t="n">
+      <c r="C15" s="33" t="n">
         <v>0.85</v>
       </c>
-      <c r="D15" s="30" t="n">
+      <c r="D15" s="33" t="n">
         <v>1.4</v>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="33" t="n">
         <v>2.55</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="31" t="inlineStr"/>
+      <c r="B17" s="34" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>ANCHORS (sourced):</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="32" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>- Retail ceiling: bulk PVA release solution ~$2.03/lb (US Composites, 20 gal) — a marked-up finished good; toll should sit below it.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="32" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>- Resin floor: PVA ~$1.38-1.60/lb (ChemAnalyst/IMARC, N.America 2026) -&gt; material ~$0.16-0.20/lb of solution.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="32" t="inlineStr">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>- Loaded contract-mfg labor ~$40/hr incl overhead; 25% margin; QC ~$30/test (cited).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="35" t="inlineStr">
         <is>
           <t>- Density ~8.5 lb/gal -&gt; 55 gal ~ 460 lb (Kuraray SG ~1.27).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="31" t="inlineStr"/>
+      <c r="B23" s="34" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>KEY CAVEAT:</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="32" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>- No public toll/per-batch rate exists. The per-batch conversion/minimum fee ($400-900/batch est.) is triangulation, NOT a citation.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="32" t="inlineStr">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>- Energy is negligible (~$3-10/batch) and materials ~$0.20/lb — do not accept these as large line items.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="32" t="inlineStr">
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>- The single biggest $/lb lever is batch size/frequency: 2 drums/batch roughly halves fixed-cost-per-lb.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="32" t="inlineStr">
+      <c r="B28" s="35" t="inlineStr">
         <is>
           <t>- Confidence: MODERATE. Pin it with 2-3 real quotes (APV / Piedmont / Columbus).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="31" t="inlineStr"/>
+      <c r="B29" s="34" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>SOURCES:</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="32" t="inlineStr">
+      <c r="B31" s="35" t="inlineStr">
         <is>
           <t>- ChemAnalyst PVA pricing: chemanalyst.com/Pricing-data/polyvinyl-alcohol-1108</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="32" t="inlineStr">
+      <c r="B32" s="35" t="inlineStr">
         <is>
           <t>- IMARC PVA pricing: imarcgroup.com/polyvinyl-alcohol-pricing-report</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="32" t="inlineStr">
+      <c r="B33" s="35" t="inlineStr">
         <is>
           <t>- US Composites mold release (retail comp): uscomposites.com/moldrelease.html</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="32" t="inlineStr">
+      <c r="B34" s="35" t="inlineStr">
         <is>
           <t>- Fibre Glast #13 PVA release film: fibreglast.com/products/pva-release-film-13</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="32" t="inlineStr">
+      <c r="B35" s="35" t="inlineStr">
         <is>
           <t>- Contract-mfg cost-plus ($40/hr, 25% margin): blog.thedigisource.com/contract-manufacturing-cost-plus</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="32" t="inlineStr">
+      <c r="B36" s="35" t="inlineStr">
         <is>
           <t>- ITC toll blending cost factors (qualitative): itctollblenders.com/2025/11/what-are-the-main-toll-blending-cost-factors/</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="32" t="inlineStr">
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t>- Kuraray Poval physical properties (density): kuraray-poval.com (basic physical properties)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="32" t="inlineStr">
+      <c r="B38" s="35" t="inlineStr">
         <is>
           <t>- Drum LTL freight: volunteerdrum.com/drum-and-tote-shipping-costs-explained/</t>
         </is>

</xml_diff>